<commit_message>
docs: sync DataCanvas backlog artifacts
</commit_message>
<xml_diff>
--- a/docs/product/sources/working/datacanvas-backlog-draft-pshe-2026-07-08.xlsx
+++ b/docs/product/sources/working/datacanvas-backlog-draft-pshe-2026-07-08.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns7="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10911"/>
   <workbookPr/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <ns2:absPath url="/Users/s060874gmail.com/coding/projects/datacanvas-first-universal-documentation-run/docs/product/sources/working/"/>
+      <x15ac:absPath url="/Users/23090718/Documents/projects/data-canvas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DDCE00D-CED2-7442-9A5C-C33788BB3E8D}" ns4:coauthVersionLast="47" ns4:coauthVersionMax="47" ns5:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DDCE00D-CED2-7442-9A5C-C33788BB3E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6060" yWindow="660" windowWidth="32180" windowHeight="19100" ns6:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6060" yWindow="660" windowWidth="32180" windowHeight="19100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" ns7:id="rId1"/>
+    <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Лист1!$B$3:$U$32</definedName>
@@ -21,13 +21,13 @@
   <calcPr calcId="191029"/>
   <extLst>
     <ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <ns8:calcFeatures>
-        <ns8:feature name="microsoft.com:RD"/>
-        <ns8:feature name="microsoft.com:Single"/>
-        <ns8:feature name="microsoft.com:FV"/>
-        <ns8:feature name="microsoft.com:CNMTM"/>
-        <ns8:feature name="microsoft.com:LET_WF"/>
-      </ns8:calcFeatures>
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -857,10 +857,10 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:U32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="40" defaultRowHeight="16" ns3:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="40" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.6640625" style="1" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="27.83203125" style="1" bestFit="1" customWidth="1"/>
@@ -882,7 +882,7 @@
     <col min="22" max="16384" width="40" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="34" ns3:dyDescent="0.2">
+    <row r="1" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="C1" s="10">
         <v>2</v>
       </c>
@@ -952,7 +952,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="34" ns3:dyDescent="0.2">
+    <row r="2" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="B2" s="17" t="s">
         <v>13</v>
       </c>
@@ -1022,7 +1022,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="3" spans="1:21" s="2" customFormat="1" ht="34" ns3:dyDescent="0.2">
+    <row r="3" spans="1:21" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
       <c r="C3" s="8" t="s">
@@ -1081,7 +1081,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="51" hidden="1" ns3:dyDescent="0.2">
+    <row r="4" spans="1:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="B4" s="17" t="s">
         <v>13</v>
       </c>
@@ -1134,7 +1134,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="51" hidden="1" ns3:dyDescent="0.2">
+    <row r="5" spans="1:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="B5" s="17" t="s">
         <v>13</v>
       </c>
@@ -1183,7 +1183,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="51" hidden="1" ns3:dyDescent="0.2">
+    <row r="6" spans="1:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="B6" s="17" t="s">
         <v>13</v>
       </c>
@@ -1229,7 +1229,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="51" hidden="1" ns3:dyDescent="0.2">
+    <row r="7" spans="1:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="B7" s="17" t="s">
         <v>13</v>
       </c>
@@ -1275,7 +1275,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="68" hidden="1" ns3:dyDescent="0.2">
+    <row r="8" spans="1:21" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="B8" s="17" t="s">
         <v>13</v>
       </c>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="U8" s="3"/>
     </row>
-    <row r="9" spans="1:21" ht="51" hidden="1" customHeight="1" ns3:dyDescent="0.2">
+    <row r="9" spans="1:21" ht="51" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="17" t="s">
         <v>13</v>
       </c>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="U9" s="3"/>
     </row>
-    <row r="10" spans="1:21" ht="102" hidden="1" ns3:dyDescent="0.2">
+    <row r="10" spans="1:21" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="B10" s="17" t="s">
         <v>13</v>
       </c>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="U10" s="3"/>
     </row>
-    <row r="11" spans="1:21" ht="34" hidden="1" ns3:dyDescent="0.2">
+    <row r="11" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="B11" s="17" t="s">
         <v>13</v>
       </c>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="U11" s="3"/>
     </row>
-    <row r="12" spans="1:21" ht="68" ns3:dyDescent="0.2">
+    <row r="12" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="B12" s="17" t="s">
         <v>13</v>
       </c>
@@ -1506,7 +1506,7 @@
       </c>
       <c r="U12" s="3"/>
     </row>
-    <row r="13" spans="1:21" ht="51" hidden="1" ns3:dyDescent="0.2">
+    <row r="13" spans="1:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="B13" s="17"/>
       <c r="C13" s="18" t="s">
         <v>39</v>
@@ -1548,7 +1548,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="51" hidden="1" ns3:dyDescent="0.2">
+    <row r="14" spans="1:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="B14" s="17"/>
       <c r="C14" s="18" t="s">
         <v>39</v>
@@ -1590,7 +1590,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="68" hidden="1" ns3:dyDescent="0.2">
+    <row r="15" spans="1:21" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="B15" s="17"/>
       <c r="C15" s="1" t="s">
         <v>14</v>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="U15" s="3"/>
     </row>
-    <row r="16" spans="1:21" ht="68" hidden="1" ns3:dyDescent="0.2">
+    <row r="16" spans="1:21" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="B16" s="17"/>
       <c r="C16" s="1" t="s">
         <v>19</v>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="U16" s="3"/>
     </row>
-    <row r="17" spans="2:21" ht="34" hidden="1" ns3:dyDescent="0.2">
+    <row r="17" spans="2:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="B17" s="17"/>
       <c r="C17" s="1" t="s">
         <v>32</v>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="U17" s="3"/>
     </row>
-    <row r="18" spans="2:21" ht="85" hidden="1" ns3:dyDescent="0.2">
+    <row r="18" spans="2:21" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="B18" s="17"/>
       <c r="C18" s="18" t="s">
         <v>39</v>
@@ -1761,7 +1761,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="19" spans="2:21" ht="34" hidden="1" ns3:dyDescent="0.2">
+    <row r="19" spans="2:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="B19" s="17"/>
       <c r="C19" s="1" t="s">
         <v>41</v>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="U19" s="3"/>
     </row>
-    <row r="20" spans="2:21" ht="51" hidden="1" ns3:dyDescent="0.2">
+    <row r="20" spans="2:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="B20" s="17"/>
       <c r="C20" s="1" t="s">
         <v>46</v>
@@ -1857,7 +1857,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="2:21" ht="51" hidden="1" ns3:dyDescent="0.2">
+    <row r="21" spans="2:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="B21" s="17"/>
       <c r="C21" s="1" t="s">
         <v>26</v>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="U21" s="3"/>
     </row>
-    <row r="22" spans="2:21" ht="51" hidden="1" ns3:dyDescent="0.2">
+    <row r="22" spans="2:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="B22" s="17"/>
       <c r="C22" s="1" t="s">
         <v>29</v>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="U22" s="3"/>
     </row>
-    <row r="23" spans="2:21" ht="51" hidden="1" ns3:dyDescent="0.2">
+    <row r="23" spans="2:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="B23" s="17"/>
       <c r="C23" s="1" t="s">
         <v>37</v>
@@ -1996,7 +1996,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="2:21" ht="68" hidden="1" ns3:dyDescent="0.2">
+    <row r="24" spans="2:21" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="B24" s="17"/>
       <c r="C24" s="1" t="s">
         <v>30</v>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="U24" s="3"/>
     </row>
-    <row r="25" spans="2:21" ht="51" hidden="1" ns3:dyDescent="0.2">
+    <row r="25" spans="2:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="B25" s="17"/>
       <c r="C25" s="1" t="s">
         <v>43</v>
@@ -2092,7 +2092,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="2:21" ht="85" ns3:dyDescent="0.2">
+    <row r="26" spans="2:21" ht="85" x14ac:dyDescent="0.2">
       <c r="B26" s="17" t="s">
         <v>77</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>65</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G26" s="6" t="s">
         <v>66</v>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="U26" s="3"/>
     </row>
-    <row r="27" spans="2:21" ht="85" ns3:dyDescent="0.2">
+    <row r="27" spans="2:21" ht="85" x14ac:dyDescent="0.2">
       <c r="B27" s="17" t="s">
         <v>78</v>
       </c>
@@ -2159,7 +2159,7 @@
         <v>68</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>66</v>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="U27" s="3"/>
     </row>
-    <row r="28" spans="2:21" ht="102" ns3:dyDescent="0.2">
+    <row r="28" spans="2:21" ht="102" x14ac:dyDescent="0.2">
       <c r="B28" s="17" t="s">
         <v>79</v>
       </c>
@@ -2210,7 +2210,7 @@
         <v>70</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G28" s="6" t="s">
         <v>66</v>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="U28" s="3"/>
     </row>
-    <row r="29" spans="2:21" ht="85" ns3:dyDescent="0.2">
+    <row r="29" spans="2:21" ht="85" x14ac:dyDescent="0.2">
       <c r="B29" s="17" t="s">
         <v>80</v>
       </c>
@@ -2292,7 +2292,7 @@
       </c>
       <c r="U29" s="3"/>
     </row>
-    <row r="30" spans="2:21" ht="102" ns3:dyDescent="0.2">
+    <row r="30" spans="2:21" ht="102" x14ac:dyDescent="0.2">
       <c r="B30" s="17" t="s">
         <v>79</v>
       </c>
@@ -2306,13 +2306,13 @@
         <v>74</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G30" s="19" t="s">
         <v>66</v>
       </c>
       <c r="H30" s="11">
-        <f>SUM(I30:U30)*$C$1</f>
+        <f t="shared" si="2"/>
         <v>26</v>
       </c>
       <c r="I30" s="16">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="U30" s="3"/>
     </row>
-    <row r="31" spans="2:21" ht="119" ns3:dyDescent="0.2">
+    <row r="31" spans="2:21" ht="119" x14ac:dyDescent="0.2">
       <c r="B31" s="17" t="s">
         <v>81</v>
       </c>
@@ -2359,7 +2359,7 @@
         <v>76</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G31" s="19" t="s">
         <v>66</v>
@@ -2394,7 +2394,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="32" spans="2:21" ht="102" ns3:dyDescent="0.2">
+    <row r="32" spans="2:21" ht="102" x14ac:dyDescent="0.2">
       <c r="B32" s="17" t="s">
         <v>96</v>
       </c>
@@ -2442,7 +2442,7 @@
       <c r="U32" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="B3:U32" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="B3:U32" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="4">
       <filters>
         <filter val="P1"/>
@@ -2452,6 +2452,6 @@
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <legacyDrawing ns4:id="rId1"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(product): align CO-002 artifact cascade
Synchronize the accepted delivery routes, priorities, resource workbook, backlog, requirements, BMC, Vision, and analysis evidence. Add a business claim map and shared public-language checks so accepted change orders remain traceable across human-readable artifacts.
</commit_message>
<xml_diff>
--- a/docs/product/sources/working/datacanvas-backlog-draft-pshe-2026-07-08.xlsx
+++ b/docs/product/sources/working/datacanvas-backlog-draft-pshe-2026-07-08.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10911"/>
   <workbookPr/>
-  <mc:AlternateContent>
-    <mc:Choice Requires="x15">
-      <x15ac:absPath url="/Users/23090718/Documents/projects/data-canvas/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DDCE00D-CED2-7442-9A5C-C33788BB3E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6060" yWindow="660" windowWidth="32180" windowHeight="19100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -16,7 +11,7 @@
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Лист1!$B$3:$U$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Лист1!$B$3:$U$36</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -153,7 +148,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="121">
   <si>
     <t>Название Story</t>
   </si>
@@ -453,6 +448,69 @@
   </si>
   <si>
     <t>Это позволит пользователю получить рабочий материал без ручной сборки презентации.</t>
+  </si>
+  <si>
+    <t>Как вызывающий агент, я хочу передавать DataCanvas входной пакет с задачей, источником запроса, параметрами презентации и данными для определения получателя результата, чтобы DataCanvas получил полный контекст запуска в проверяемом формате.</t>
+  </si>
+  <si>
+    <t>Это снижает риск неполного или неоднозначного запуска презентации и ошибочной доставки результата.</t>
+  </si>
+  <si>
+    <t>Как вызывающий агент, я хочу получать от DataCanvas сообщение о приеме данных, статусы обработки и сведения о результате, чтобы понимать, принят ли запрос, требуется ли уточнение и завершилась ли подготовка презентации.</t>
+  </si>
+  <si>
+    <t>Это позволяет другому агенту корректно вести общий сценарий и не терять состояние задачи; готовый результат доставляется пользователю по электронной почте.</t>
+  </si>
+  <si>
+    <t>Как команда разработки, мы хотим сохранять проверяемую связь между источником запроса, результатом проверки входа, статусами обработки и итоговыми файлами, чтобы каждый запуск DataCanvas другим агентом был проверяемым и воспроизводимым.</t>
+  </si>
+  <si>
+    <t>Проверяемость маршрута</t>
+  </si>
+  <si>
+    <t>Как DataCanvas, я хочу сформировать редактируемый `PPTX`-файл презентации и нередактируемую `PDF`-копию из уже проверенных и нормализованных данных, чтобы пользователь получил рабочий материал без ручной сборки.</t>
+  </si>
+  <si>
+    <t>Это позволит пользователю получить рабочий материал без ручной сборки презентации и иметь нередактируемую копию для просмотра или передачи.</t>
+  </si>
+  <si>
+    <t>Как DataCanvas, я хочу отправлять созданные файлы презентации по электронной почте в разрешенные рабочие контуры, чтобы пользователь получал результат там, где с ним можно безопасно работать.</t>
+  </si>
+  <si>
+    <t>Расширенная доставка</t>
+  </si>
+  <si>
+    <t>Это позволит расширить доставку результата без ручной пересылки между рабочими контурами.</t>
+  </si>
+  <si>
+    <t>Как DataCanvas, я хочу сохранять нередактируемую `PDF`-копию презентации в защищенном хранилище, чтобы результат можно было открыть по ссылке без повторной отправки файла.</t>
+  </si>
+  <si>
+    <t>Хранение результата</t>
+  </si>
+  <si>
+    <t>Это позволит безопасно переиспользовать готовую копию результата после генерации.</t>
+  </si>
+  <si>
+    <t>Как вызывающий агент, я хочу получать от DataCanvas ссылку на нередактируемую `PDF`-копию, чтобы передать пользователю доступ к готовому результату в своем сценарии.</t>
+  </si>
+  <si>
+    <t>Передача ссылки</t>
+  </si>
+  <si>
+    <t>Это позволит другому агенту продолжить сценарий после подготовки презентации и не пересылать сам файл.</t>
+  </si>
+  <si>
+    <t>Как пользователь Лисы, я хочу</t>
+  </si>
+  <si>
+    <t>Как пользователь Лисы, я хочу получать ссылку на готовую презентацию и уведомление о готовности через сценарий, который ведут вызывающий агент и Лиса, чтобы открыть результат из текущего рабочего контекста.</t>
+  </si>
+  <si>
+    <t>Уведомление в Лисе</t>
+  </si>
+  <si>
+    <t>Это позволит пользователю быстрее перейти от уведомления к готовой презентации без поиска письма или файла.</t>
   </si>
 </sst>
 </file>
@@ -859,7 +917,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:U32"/>
+  <dimension ref="A1:U36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="40" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.6640625" style="1" hidden="1" customWidth="1"/>
@@ -888,28 +946,28 @@
       </c>
       <c r="D1" s="12">
         <f>SUM(I1,Q1:T1)</f>
-        <v>156</v>
+        <v>224</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>59</v>
       </c>
       <c r="F1" s="12">
         <f>SUM(I1:U1)</f>
-        <v>179.4</v>
+        <v>289.8</v>
       </c>
       <c r="G1" s="12"/>
       <c r="H1" s="12"/>
       <c r="I1" s="15">
         <f t="shared" ref="I1:U1" si="0">I2*$C$1</f>
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="J1" s="13">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K1" s="13">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L1" s="13">
         <f t="shared" si="0"/>
@@ -921,35 +979,35 @@
       </c>
       <c r="N1" s="13">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="O1" s="13">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P1" s="13">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q1" s="14">
         <f t="shared" si="0"/>
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="R1" s="14">
         <f t="shared" si="0"/>
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="S1" s="14">
         <f t="shared" si="0"/>
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="T1" s="14">
         <f t="shared" si="0"/>
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="U1" s="13">
         <f t="shared" si="0"/>
-        <v>1.4</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="34" x14ac:dyDescent="0.2">
@@ -958,28 +1016,28 @@
       </c>
       <c r="D2" s="12">
         <f>SUM(I2,Q2:T2)</f>
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>58</v>
       </c>
       <c r="F2" s="12">
         <f>SUM(I2:U2)</f>
-        <v>89.7</v>
+        <v>144.9</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="12"/>
       <c r="I2" s="14">
         <f t="shared" ref="I2:U2" si="1">SUBTOTAL(9,I$4:I$500)</f>
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="J2" s="13">
         <f t="shared" si="1"/>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="K2" s="13">
         <f t="shared" si="1"/>
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="L2" s="13">
         <f t="shared" si="1"/>
@@ -991,35 +1049,35 @@
       </c>
       <c r="N2" s="13">
         <f t="shared" si="1"/>
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="O2" s="13">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="P2" s="13">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="Q2" s="14">
         <f t="shared" si="1"/>
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="R2" s="14">
         <f t="shared" si="1"/>
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="S2" s="14">
         <f t="shared" si="1"/>
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="T2" s="14">
         <f t="shared" si="1"/>
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="U2" s="13">
         <f t="shared" si="1"/>
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="3" spans="1:21" s="2" customFormat="1" ht="34" x14ac:dyDescent="0.2">
@@ -1154,7 +1212,7 @@
         <v>90</v>
       </c>
       <c r="H5" s="11">
-        <f t="shared" ref="H5:H32" si="2">SUM(I5:U5)*$C$1</f>
+        <f t="shared" ref="H5:H36" si="2">SUM(I5:U5)*$C$1</f>
         <v>13.4</v>
       </c>
       <c r="I5" s="16">
@@ -2201,13 +2259,13 @@
         <v>79</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>92</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>70</v>
+        <v>101</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>49</v>
@@ -2297,13 +2355,13 @@
         <v>79</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>94</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>49</v>
@@ -2350,10 +2408,10 @@
         <v>81</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>75</v>
+        <v>104</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>76</v>
@@ -2399,13 +2457,13 @@
         <v>96</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>98</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>49</v>
@@ -2441,8 +2499,230 @@
       </c>
       <c r="U32" s="3"/>
     </row>
+    <row r="33" spans="2:21" ht="102" x14ac:dyDescent="0.2">
+      <c r="B33" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G33" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="H33" s="11">
+        <f t="shared" si="2"/>
+        <v>26</v>
+      </c>
+      <c r="I33" s="16">
+        <v>1</v>
+      </c>
+      <c r="J33" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="K33" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="L33" s="3"/>
+      <c r="M33" s="3"/>
+      <c r="N33" s="3">
+        <v>3</v>
+      </c>
+      <c r="O33" s="3"/>
+      <c r="P33" s="3"/>
+      <c r="Q33" s="16">
+        <v>2</v>
+      </c>
+      <c r="R33" s="16">
+        <v>2</v>
+      </c>
+      <c r="S33" s="16">
+        <v>2</v>
+      </c>
+      <c r="T33" s="16">
+        <v>2</v>
+      </c>
+      <c r="U33" s="3"/>
+    </row>
+    <row r="34" spans="2:21" ht="102" x14ac:dyDescent="0.2">
+      <c r="B34" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G34" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="H34" s="11">
+        <f t="shared" si="2"/>
+        <v>27.4</v>
+      </c>
+      <c r="I34" s="16">
+        <v>1</v>
+      </c>
+      <c r="J34" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="K34" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="L34" s="3"/>
+      <c r="M34" s="3"/>
+      <c r="N34" s="3">
+        <v>3</v>
+      </c>
+      <c r="O34" s="3"/>
+      <c r="P34" s="3"/>
+      <c r="Q34" s="16">
+        <v>2</v>
+      </c>
+      <c r="R34" s="16">
+        <v>2</v>
+      </c>
+      <c r="S34" s="16">
+        <v>2</v>
+      </c>
+      <c r="T34" s="16">
+        <v>2</v>
+      </c>
+      <c r="U34" s="3">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="35" spans="2:21" ht="102" x14ac:dyDescent="0.2">
+      <c r="B35" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G35" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="H35" s="11">
+        <f t="shared" si="2"/>
+        <v>28</v>
+      </c>
+      <c r="I35" s="16">
+        <v>1</v>
+      </c>
+      <c r="J35" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="K35" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="L35" s="3"/>
+      <c r="M35" s="3"/>
+      <c r="N35" s="3">
+        <v>2</v>
+      </c>
+      <c r="O35" s="3">
+        <v>1</v>
+      </c>
+      <c r="P35" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q35" s="16">
+        <v>2</v>
+      </c>
+      <c r="R35" s="16">
+        <v>2</v>
+      </c>
+      <c r="S35" s="16">
+        <v>2</v>
+      </c>
+      <c r="T35" s="16">
+        <v>2</v>
+      </c>
+      <c r="U35" s="3"/>
+    </row>
+    <row r="36" spans="2:21" ht="102" x14ac:dyDescent="0.2">
+      <c r="B36" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G36" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="H36" s="11">
+        <f t="shared" si="2"/>
+        <v>29</v>
+      </c>
+      <c r="I36" s="16">
+        <v>1</v>
+      </c>
+      <c r="J36" s="3">
+        <v>1</v>
+      </c>
+      <c r="K36" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="L36" s="3"/>
+      <c r="M36" s="3"/>
+      <c r="N36" s="3">
+        <v>3</v>
+      </c>
+      <c r="O36" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="P36" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="Q36" s="16">
+        <v>1</v>
+      </c>
+      <c r="R36" s="16">
+        <v>1</v>
+      </c>
+      <c r="S36" s="16">
+        <v>2</v>
+      </c>
+      <c r="T36" s="16">
+        <v>2</v>
+      </c>
+      <c r="U36" s="3"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B3:U32" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="B3:U36" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="4">
       <filters>
         <filter val="P1"/>

</xml_diff>